<commit_message>
fixes to access control and adding test guide
</commit_message>
<xml_diff>
--- a/docs/bunnywell-database-cleanup-template-v2.xlsx
+++ b/docs/bunnywell-database-cleanup-template-v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlg\Documents\GitHub\Bunnywell_Portal\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8DF9338-8D82-4F3F-9E47-F4987F000978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758C9BC0-5F0A-4F84-A437-9A8A37CE5A4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13866" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1620" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1624" uniqueCount="220">
   <si>
     <t>Bunnywell Database Cleanup Template</t>
   </si>
@@ -697,13 +697,22 @@
   </si>
   <si>
     <t>07826 875941</t>
+  </si>
+  <si>
+    <t>carl.gilbert@gmail.com</t>
+  </si>
+  <si>
+    <t>Carl Gilbert</t>
+  </si>
+  <si>
+    <t>Staging admin</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -730,6 +739,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -786,10 +801,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -810,8 +826,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1023,17 +1042,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="20.25">
+    <row r="1" spans="1:1" ht="20">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="28.5">
+    <row r="3" spans="1:1" ht="27.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1085,8 +1104,8 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -1097,7 +1116,7 @@
     <col min="7" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" ht="14">
       <c r="A1" s="10" t="s">
         <v>104</v>
       </c>
@@ -1109,7 +1128,7 @@
       <c r="G1" s="11"/>
       <c r="H1" s="11"/>
     </row>
-    <row r="3" spans="1:8" ht="15">
+    <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
         <v>97</v>
       </c>
@@ -1219,12 +1238,30 @@
       </c>
       <c r="H7" t="s">
         <v>197</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="B8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C8" t="s">
+        <v>110</v>
+      </c>
+      <c r="F8" s="13"/>
+      <c r="H8" t="s">
+        <v>219</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A8" r:id="rId1" xr:uid="{0E35F4FA-BC1A-4699-944C-9066C85EB0C6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1232,7 +1269,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -1242,7 +1279,7 @@
     <col min="7" max="7" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" ht="14">
       <c r="A1" s="10" t="s">
         <v>115</v>
       </c>
@@ -1253,7 +1290,7 @@
       <c r="F1" s="11"/>
       <c r="G1" s="11"/>
     </row>
-    <row r="3" spans="1:7" ht="15">
+    <row r="3" spans="1:7">
       <c r="A3" s="4" t="s">
         <v>116</v>
       </c>
@@ -1385,7 +1422,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="2" width="17" customWidth="1"/>
     <col min="3" max="4" width="18" customWidth="1"/>
@@ -1395,7 +1432,7 @@
     <col min="10" max="10" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" ht="14">
       <c r="A1" s="10" t="s">
         <v>10</v>
       </c>
@@ -1409,7 +1446,7 @@
       <c r="I1" s="11"/>
       <c r="J1" s="11"/>
     </row>
-    <row r="3" spans="1:10" ht="15">
+    <row r="3" spans="1:10">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -1511,7 +1548,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -1520,7 +1557,7 @@
     <col min="5" max="5" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="14">
       <c r="A1" s="10" t="s">
         <v>24</v>
       </c>
@@ -1529,7 +1566,7 @@
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
     </row>
-    <row r="3" spans="1:5" ht="15">
+    <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
         <v>25</v>
       </c>
@@ -1633,7 +1670,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -1643,7 +1680,7 @@
     <col min="6" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" ht="14">
       <c r="A1" s="10" t="s">
         <v>41</v>
       </c>
@@ -1653,7 +1690,7 @@
       <c r="E1" s="11"/>
       <c r="F1" s="11"/>
     </row>
-    <row r="3" spans="1:6" ht="15">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>27</v>
       </c>
@@ -2061,7 +2098,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:O152"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -2077,7 +2114,7 @@
     <col min="15" max="15" width="33" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" ht="14">
       <c r="A1" s="10" t="s">
         <v>58</v>
       </c>
@@ -2096,7 +2133,7 @@
       <c r="N1" s="11"/>
       <c r="O1" s="11"/>
     </row>
-    <row r="3" spans="1:15" ht="15">
+    <row r="3" spans="1:15">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -7621,7 +7658,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -7640,7 +7677,7 @@
       <c r="E1" s="11"/>
       <c r="F1" s="11"/>
     </row>
-    <row r="3" spans="1:6" ht="15">
+    <row r="3" spans="1:6">
       <c r="A3" s="4" t="s">
         <v>11</v>
       </c>
@@ -7871,15 +7908,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E73"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="21.125" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" customWidth="1"/>
     <col min="3" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="14">
       <c r="A1" s="10" t="s">
         <v>91</v>
       </c>
@@ -7888,7 +7925,7 @@
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
     </row>
-    <row r="3" spans="1:5" ht="15">
+    <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -8899,16 +8936,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
-    <col min="4" max="4" width="27.125" customWidth="1"/>
+    <col min="4" max="4" width="27.109375" customWidth="1"/>
     <col min="5" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" ht="14">
       <c r="A1" s="10" t="s">
         <v>93</v>
       </c>
@@ -8918,7 +8955,7 @@
       <c r="E1" s="11"/>
       <c r="F1" s="11"/>
     </row>
-    <row r="3" spans="1:6" ht="15">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>94</v>
       </c>
@@ -9018,21 +9055,21 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.7"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" ht="14">
       <c r="A1" s="10" t="s">
         <v>102</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
     </row>
-    <row r="3" spans="1:3" ht="15">
+    <row r="3" spans="1:3">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>

</xml_diff>